<commit_message>
SS and SL models
Minor code updates for SS and SL final model outputs
</commit_message>
<xml_diff>
--- a/Data layers/Important_locations.xlsx
+++ b/Data layers/Important_locations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Williams\Documents\GitHub\HSM-and-mapping\Data layers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B94CAB3E-C81E-4728-BF5E-AF4D933EB5A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F68B8B-0787-415B-9FA6-6356E7C9D8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CA14E8E-9857-4D7B-B94E-961384FE881B}"/>
+    <workbookView xWindow="1632" yWindow="2820" windowWidth="17280" windowHeight="8928" xr2:uid="{2CA14E8E-9857-4D7B-B94E-961384FE881B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>Longitude</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>STL-STPT</t>
+  </si>
+  <si>
+    <t>USGS-02313700</t>
   </si>
 </sst>
 </file>
@@ -495,10 +498,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02EA6A26-70AD-4971-B57D-DACA2AD4442C}">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -512,7 +519,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>-82.720104000000006</v>
       </c>
@@ -526,7 +533,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>-83.142859999999999</v>
       </c>
@@ -540,7 +547,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>-83.377600000000001</v>
       </c>
@@ -554,7 +561,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>-83.288775999999999</v>
       </c>
@@ -568,7 +575,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>-83.034009999999995</v>
       </c>
@@ -582,7 +589,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>-82.621020000000001</v>
       </c>
@@ -596,7 +603,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>-80.254469999999998</v>
       </c>
@@ -610,7 +617,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>-83.086667000000006</v>
       </c>
@@ -624,7 +631,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>-82.617926267019001</v>
       </c>
@@ -638,7 +645,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>-83.162099999999995</v>
       </c>
@@ -652,7 +659,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>-83.062749999999994</v>
       </c>
@@ -666,7 +673,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>-83.241699999999994</v>
       </c>
@@ -680,7 +687,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>-83.341700000000003</v>
       </c>
@@ -694,7 +701,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>-83.022779999999997</v>
       </c>
@@ -708,7 +715,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>-80.359804999999994</v>
       </c>
@@ -722,7 +729,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>-80.285263</v>
       </c>
@@ -736,7 +743,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>-80.34066</v>
       </c>
@@ -750,7 +757,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>-80.288118999999995</v>
       </c>
@@ -764,7 +771,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>-80.258364</v>
       </c>
@@ -778,7 +785,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>-80.207002000000003</v>
       </c>
@@ -790,6 +797,20 @@
       </c>
       <c r="D21" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>-82.769001071597003</v>
+      </c>
+      <c r="B22" s="1">
+        <v>29.204133775691599</v>
+      </c>
+      <c r="C22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>